<commit_message>
fix units, remove old files
</commit_message>
<xml_diff>
--- a/InputData/elec/FoGBPD/Fraction of Grid Batteries Produced Domestically.xlsx
+++ b/InputData/elec/FoGBPD/Fraction of Grid Batteries Produced Domestically.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28906"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skorpius/My Drive/2024/FO local_EPS ICM/Diario/20250423_Last 50/FoGBPD/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\elec\FoGBPD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C29CF46-7C87-794B-8935-C9E2B51274C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B596E9B9-CA74-4146-839D-31FF75B6C6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="4" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -154,7 +154,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,14 +243,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -258,16 +255,20 @@
     <xf numFmtId="9" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -541,9 +542,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -581,7 +582,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -687,7 +688,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -829,7 +830,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -838,175 +839,175 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF982137-6F01-4109-8226-D4C6F3731BA9}">
   <dimension ref="A1:B34"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="101.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
         <v>2023</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="2">
         <v>2024</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="2">
         <v>2024</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="2">
         <v>2024</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>22</v>
       </c>
@@ -1019,14 +1020,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8456871-96FC-47A8-BE1A-65358738DEAC}">
   <dimension ref="L2:O33"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="12:14">
+    <row r="2" spans="12:14" x14ac:dyDescent="0.25">
       <c r="L2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="12:14">
+    <row r="3" spans="12:14" x14ac:dyDescent="0.25">
       <c r="L3">
         <v>2022</v>
       </c>
@@ -1037,7 +1038,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="12:14">
+    <row r="4" spans="12:14" x14ac:dyDescent="0.25">
       <c r="L4">
         <v>2030</v>
       </c>
@@ -1048,12 +1049,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="12:15">
+    <row r="21" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="12:15">
+    <row r="22" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L22">
         <v>2022</v>
       </c>
@@ -1064,7 +1065,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="12:15">
+    <row r="23" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L23">
         <v>2030</v>
       </c>
@@ -1078,35 +1079,35 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="12:15">
+    <row r="25" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L25" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="12:15">
+    <row r="26" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L26">
         <v>2030</v>
       </c>
-      <c r="M26" s="4">
+      <c r="M26" s="3">
         <f>0.1+0.1/0.75*0.25</f>
         <v>0.13333333333333333</v>
       </c>
     </row>
-    <row r="27" spans="12:15">
-      <c r="L27" s="5" t="s">
+    <row r="27" spans="12:15" x14ac:dyDescent="0.25">
+      <c r="L27" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="12:15">
+    <row r="29" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L29" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="12:15">
+    <row r="30" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L30">
         <v>2030</v>
       </c>
-      <c r="M30" s="6">
+      <c r="M30" s="5">
         <f>M23*M26</f>
         <v>103.06666666666666</v>
       </c>
@@ -1114,16 +1115,16 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="12:15">
+    <row r="32" spans="12:15" x14ac:dyDescent="0.25">
       <c r="L32" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="12:13">
+    <row r="33" spans="12:13" x14ac:dyDescent="0.25">
       <c r="L33">
         <v>2030</v>
       </c>
-      <c r="M33" s="7">
+      <c r="M33" s="6">
         <f>M30/M4</f>
         <v>0.86610644257703073</v>
       </c>
@@ -1137,14 +1138,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B49FB018-EAB2-4AB3-B95C-024DA6C229C7}">
   <dimension ref="J6:O32"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="6" spans="14:15">
+    <row r="6" spans="14:15" x14ac:dyDescent="0.25">
       <c r="N6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="14:15">
+    <row r="7" spans="14:15" x14ac:dyDescent="0.25">
       <c r="N7">
         <v>2022</v>
       </c>
@@ -1153,7 +1154,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="14:15">
+    <row r="8" spans="14:15" x14ac:dyDescent="0.25">
       <c r="N8">
         <v>2030</v>
       </c>
@@ -1162,12 +1163,12 @@
         <v>110</v>
       </c>
     </row>
-    <row r="27" spans="10:12">
+    <row r="27" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="10:12">
+    <row r="28" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J28">
         <v>2022</v>
       </c>
@@ -1179,7 +1180,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="10:12">
+    <row r="29" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J29">
         <v>2030</v>
       </c>
@@ -1190,16 +1191,16 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="10:12">
+    <row r="31" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J31" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="10:12">
+    <row r="32" spans="10:12" x14ac:dyDescent="0.25">
       <c r="J32">
         <v>2030</v>
       </c>
-      <c r="K32" s="7">
+      <c r="K32" s="6">
         <f>O8/K29</f>
         <v>0.95652173913043481</v>
       </c>
@@ -1213,20 +1214,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13AB29A9-70CB-4471-AE81-9A64EFDA202F}">
   <dimension ref="B21:B24"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="2:2">
-      <c r="B24" s="8">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="7">
         <v>0.62</v>
       </c>
     </row>
@@ -1242,319 +1243,321 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AY2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.42578125" style="9" customWidth="1"/>
+    <col min="2" max="5" width="8.85546875" style="9"/>
+    <col min="6" max="6" width="10.28515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.85546875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51">
-      <c r="A1" t="s">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B1">
+      <c r="B1" s="9">
         <v>2021</v>
       </c>
-      <c r="C1">
+      <c r="C1" s="9">
         <v>2022</v>
       </c>
-      <c r="D1">
+      <c r="D1" s="9">
         <v>2023</v>
       </c>
-      <c r="E1">
+      <c r="E1" s="9">
         <v>2024</v>
       </c>
-      <c r="F1">
+      <c r="F1" s="9">
         <v>2025</v>
       </c>
-      <c r="G1">
+      <c r="G1" s="9">
         <v>2026</v>
       </c>
-      <c r="H1">
+      <c r="H1" s="9">
         <v>2027</v>
       </c>
-      <c r="I1">
+      <c r="I1" s="9">
         <v>2028</v>
       </c>
-      <c r="J1">
+      <c r="J1" s="9">
         <v>2029</v>
       </c>
-      <c r="K1">
+      <c r="K1" s="9">
         <v>2030</v>
       </c>
-      <c r="L1">
+      <c r="L1" s="9">
         <v>2031</v>
       </c>
-      <c r="M1">
+      <c r="M1" s="9">
         <v>2032</v>
       </c>
-      <c r="N1">
+      <c r="N1" s="9">
         <v>2033</v>
       </c>
-      <c r="O1">
+      <c r="O1" s="9">
         <v>2034</v>
       </c>
-      <c r="P1">
+      <c r="P1" s="9">
         <v>2035</v>
       </c>
-      <c r="Q1">
+      <c r="Q1" s="9">
         <v>2036</v>
       </c>
-      <c r="R1">
+      <c r="R1" s="9">
         <v>2037</v>
       </c>
-      <c r="S1">
+      <c r="S1" s="9">
         <v>2038</v>
       </c>
-      <c r="T1">
+      <c r="T1" s="9">
         <v>2039</v>
       </c>
-      <c r="U1">
+      <c r="U1" s="9">
         <v>2040</v>
       </c>
-      <c r="V1">
+      <c r="V1" s="9">
         <v>2041</v>
       </c>
-      <c r="W1">
+      <c r="W1" s="9">
         <v>2042</v>
       </c>
-      <c r="X1">
+      <c r="X1" s="9">
         <v>2043</v>
       </c>
-      <c r="Y1">
+      <c r="Y1" s="9">
         <v>2044</v>
       </c>
-      <c r="Z1">
+      <c r="Z1" s="9">
         <v>2045</v>
       </c>
-      <c r="AA1">
+      <c r="AA1" s="9">
         <v>2046</v>
       </c>
-      <c r="AB1">
+      <c r="AB1" s="9">
         <v>2047</v>
       </c>
-      <c r="AC1">
+      <c r="AC1" s="9">
         <v>2048</v>
       </c>
-      <c r="AD1">
+      <c r="AD1" s="9">
         <v>2049</v>
       </c>
-      <c r="AE1">
+      <c r="AE1" s="9">
         <v>2050</v>
       </c>
-      <c r="AF1">
+      <c r="AF1" s="9">
         <v>2051</v>
       </c>
-      <c r="AG1">
+      <c r="AG1" s="9">
         <v>2052</v>
       </c>
-      <c r="AH1">
+      <c r="AH1" s="9">
         <v>2053</v>
       </c>
-      <c r="AI1">
+      <c r="AI1" s="9">
         <v>2054</v>
       </c>
-      <c r="AJ1">
+      <c r="AJ1" s="9">
         <v>2055</v>
       </c>
-      <c r="AK1">
+      <c r="AK1" s="9">
         <v>2056</v>
       </c>
-      <c r="AL1">
+      <c r="AL1" s="9">
         <v>2057</v>
       </c>
-      <c r="AM1">
+      <c r="AM1" s="9">
         <v>2058</v>
       </c>
-      <c r="AN1">
+      <c r="AN1" s="9">
         <v>2059</v>
       </c>
-      <c r="AO1">
+      <c r="AO1" s="9">
         <v>2060</v>
       </c>
-      <c r="AP1">
+      <c r="AP1" s="9">
         <v>2061</v>
       </c>
-      <c r="AQ1">
+      <c r="AQ1" s="9">
         <v>2062</v>
       </c>
-      <c r="AR1">
+      <c r="AR1" s="9">
         <v>2063</v>
       </c>
-      <c r="AS1">
+      <c r="AS1" s="9">
         <v>2064</v>
       </c>
-      <c r="AT1">
+      <c r="AT1" s="9">
         <v>2065</v>
       </c>
-      <c r="AU1">
+      <c r="AU1" s="9">
         <v>2066</v>
       </c>
-      <c r="AV1">
+      <c r="AV1" s="9">
         <v>2067</v>
       </c>
-      <c r="AW1">
+      <c r="AW1" s="9">
         <v>2068</v>
       </c>
-      <c r="AX1">
+      <c r="AX1" s="9">
         <v>2069</v>
       </c>
-      <c r="AY1">
+      <c r="AY1" s="9">
         <v>2070</v>
       </c>
     </row>
-    <row r="2" spans="1:51" s="3" customFormat="1" ht="32.1">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:51" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="10">
-        <v>0</v>
-      </c>
-      <c r="C2" s="10">
-        <v>0</v>
-      </c>
-      <c r="D2" s="10">
-        <v>0</v>
-      </c>
-      <c r="E2" s="10">
-        <v>0</v>
-      </c>
-      <c r="F2" s="10">
-        <v>0</v>
-      </c>
-      <c r="G2" s="11">
-        <v>0</v>
-      </c>
-      <c r="H2" s="11">
-        <v>0</v>
-      </c>
-      <c r="I2" s="11">
-        <v>0</v>
-      </c>
-      <c r="J2" s="11">
-        <v>0</v>
-      </c>
-      <c r="K2" s="12">
-        <v>0</v>
-      </c>
-      <c r="L2" s="13">
-        <v>0</v>
-      </c>
-      <c r="M2" s="13">
-        <v>0</v>
-      </c>
-      <c r="N2" s="13">
-        <v>0</v>
-      </c>
-      <c r="O2" s="13">
-        <v>0</v>
-      </c>
-      <c r="P2" s="13">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="13">
-        <v>0</v>
-      </c>
-      <c r="R2" s="13">
-        <v>0</v>
-      </c>
-      <c r="S2" s="13">
-        <v>0</v>
-      </c>
-      <c r="T2" s="13">
-        <v>0</v>
-      </c>
-      <c r="U2" s="13">
-        <v>0</v>
-      </c>
-      <c r="V2" s="13">
-        <v>0</v>
-      </c>
-      <c r="W2" s="13">
-        <v>0</v>
-      </c>
-      <c r="X2" s="13">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="13">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AH2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AI2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AK2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AL2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AN2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AO2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AP2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AQ2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AR2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AS2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AT2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AU2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AV2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AW2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AX2" s="13">
-        <v>0</v>
-      </c>
-      <c r="AY2" s="13">
+      <c r="B2" s="11">
+        <v>0</v>
+      </c>
+      <c r="C2" s="11">
+        <v>0</v>
+      </c>
+      <c r="D2" s="11">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11">
+        <v>0</v>
+      </c>
+      <c r="F2" s="11">
+        <v>0</v>
+      </c>
+      <c r="G2" s="12">
+        <v>0</v>
+      </c>
+      <c r="H2" s="12">
+        <v>0</v>
+      </c>
+      <c r="I2" s="12">
+        <v>0</v>
+      </c>
+      <c r="J2" s="12">
+        <v>0</v>
+      </c>
+      <c r="K2" s="13">
+        <v>0</v>
+      </c>
+      <c r="L2" s="14">
+        <v>0</v>
+      </c>
+      <c r="M2" s="14">
+        <v>0</v>
+      </c>
+      <c r="N2" s="14">
+        <v>0</v>
+      </c>
+      <c r="O2" s="14">
+        <v>0</v>
+      </c>
+      <c r="P2" s="14">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="14">
+        <v>0</v>
+      </c>
+      <c r="R2" s="14">
+        <v>0</v>
+      </c>
+      <c r="S2" s="14">
+        <v>0</v>
+      </c>
+      <c r="T2" s="14">
+        <v>0</v>
+      </c>
+      <c r="U2" s="14">
+        <v>0</v>
+      </c>
+      <c r="V2" s="14">
+        <v>0</v>
+      </c>
+      <c r="W2" s="14">
+        <v>0</v>
+      </c>
+      <c r="X2" s="14">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="14">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AR2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AS2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AT2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AU2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AV2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AW2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AX2" s="14">
+        <v>0</v>
+      </c>
+      <c r="AY2" s="14">
         <v>0</v>
       </c>
     </row>
@@ -1708,6 +1711,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1716,20 +1725,37 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDECB4E9-2802-4981-AC9C-BF65B211447C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDECB4E9-2802-4981-AC9C-BF65B211447C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37A0FAA7-EFDF-4FEF-98FD-6C773B11E909}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0557BFBA-A71F-4522-9D29-D655DC86AFC7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0557BFBA-A71F-4522-9D29-D655DC86AFC7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37A0FAA7-EFDF-4FEF-98FD-6C773B11E909}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>